<commit_message>
Add RDS coupon analysis report & supporting files
setting up the analysis environment
</commit_message>
<xml_diff>
--- a/data/Eldoret_coupon.xlsx
+++ b/data/Eldoret_coupon.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APHRC\R_Work\CIPSE Analysis\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\GitHub\APHRC\cipse_rds_analysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4DDB8F16-1984-4290-8716-BBC10E33B724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C57D5B6-D0D1-4E67-9BAB-4F477B34B9B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CTF" sheetId="1" r:id="rId1"/>
     <sheet name="CHECK" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet name="STAT" sheetId="3" r:id="rId3"/>
-    <sheet name="About" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="About" sheetId="4" state="hidden" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,70 +34,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Coupons released to participiants</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Returned coupons (seeds excluded)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Number of non-eligible participiants</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Number of Coupons yet to be returned (valid and expired coupons)</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="458">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -1459,84 +1396,6 @@
   </si>
   <si>
     <t>Coupon 3</t>
-  </si>
-  <si>
-    <t>COUPONS STATISTICS</t>
-  </si>
-  <si>
-    <t>Coupons</t>
-  </si>
-  <si>
-    <t>Number of participiant entered into RDS study</t>
-  </si>
-  <si>
-    <t>SEED</t>
-  </si>
-  <si>
-    <t>RELEASED</t>
-  </si>
-  <si>
-    <t>RETURNED</t>
-  </si>
-  <si>
-    <t>NEL/REF</t>
-  </si>
-  <si>
-    <t>OUT</t>
-  </si>
-  <si>
-    <t>W0</t>
-  </si>
-  <si>
-    <t>W1</t>
-  </si>
-  <si>
-    <t>W2</t>
-  </si>
-  <si>
-    <t>W3</t>
-  </si>
-  <si>
-    <t>W4</t>
-  </si>
-  <si>
-    <t>W5</t>
-  </si>
-  <si>
-    <t>W6</t>
-  </si>
-  <si>
-    <t>W7</t>
-  </si>
-  <si>
-    <t>W8</t>
-  </si>
-  <si>
-    <t>W9</t>
-  </si>
-  <si>
-    <t>W10</t>
-  </si>
-  <si>
-    <t>W11</t>
-  </si>
-  <si>
-    <t>W12</t>
-  </si>
-  <si>
-    <t>W13</t>
-  </si>
-  <si>
-    <t>W14</t>
-  </si>
-  <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
-    <t>Valid participants</t>
-  </si>
-  <si>
-    <t>Non-Eligible</t>
   </si>
   <si>
     <t>Coupon Tracking Form Ver. 3.1</t>
@@ -1660,12 +1519,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="165" formatCode="&quot;RDS-&quot;####"/>
-    <numFmt numFmtId="166" formatCode="##########*0"/>
-    <numFmt numFmtId="168" formatCode="dd/mm/yyyy/"/>
-    <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="164" formatCode="&quot;RDS-&quot;####"/>
+    <numFmt numFmtId="165" formatCode="##########*0"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy/"/>
+    <numFmt numFmtId="167" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1709,17 +1568,12 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="6"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1746,12 +1600,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF99CC"/>
-        <bgColor rgb="FFFF99CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF99CC00"/>
         <bgColor rgb="FF99CC00"/>
       </patternFill>
@@ -1769,7 +1617,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="53">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -1799,17 +1647,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
@@ -1830,15 +1667,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -1849,31 +1677,6 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
@@ -1917,18 +1720,17 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -2018,183 +1820,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -2303,208 +1928,122 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="4" fillId="4" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="4" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2513,59 +2052,39 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="7" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
-    <dxf>
-      <font>
-        <color rgb="FFCCFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFDDDDDD"/>
-      </font>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-    </dxf>
+  <dxfs count="14">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2902,13 +2421,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2919,7 +2438,7 @@
       <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="6">
         <v>1</v>
       </c>
     </row>
@@ -2930,7 +2449,7 @@
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="6">
         <v>2</v>
       </c>
     </row>
@@ -2941,7 +2460,7 @@
       <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>3</v>
       </c>
     </row>
@@ -2952,7 +2471,7 @@
       <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <v>4</v>
       </c>
     </row>
@@ -2963,7 +2482,7 @@
       <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>113331</v>
       </c>
     </row>
@@ -2974,7 +2493,7 @@
       <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="7">
         <v>11111113</v>
       </c>
     </row>
@@ -2985,7 +2504,7 @@
       <c r="B8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="6">
         <v>113332</v>
       </c>
     </row>
@@ -2996,7 +2515,7 @@
       <c r="B9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="6">
         <v>11</v>
       </c>
     </row>
@@ -3007,7 +2526,7 @@
       <c r="B10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="6">
         <v>11133</v>
       </c>
     </row>
@@ -3018,7 +2537,7 @@
       <c r="B11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="6">
         <v>111123</v>
       </c>
     </row>
@@ -3029,7 +2548,7 @@
       <c r="B12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="6">
         <v>11112231</v>
       </c>
     </row>
@@ -3040,7 +2559,7 @@
       <c r="B13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="6">
         <v>1111223232</v>
       </c>
     </row>
@@ -3051,7 +2570,7 @@
       <c r="B14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="6">
         <v>113223213</v>
       </c>
     </row>
@@ -3062,7 +2581,7 @@
       <c r="B15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="6">
         <v>1132233</v>
       </c>
     </row>
@@ -3073,7 +2592,7 @@
       <c r="B16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="6">
         <v>113222</v>
       </c>
     </row>
@@ -3084,7 +2603,7 @@
       <c r="B17" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="6">
         <v>11323</v>
       </c>
     </row>
@@ -4217,7 +3736,7 @@
       <c r="B120" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C120" s="9">
+      <c r="C120" s="8">
         <v>21632</v>
       </c>
     </row>
@@ -4767,7 +4286,7 @@
       <c r="B170" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="C170" s="9">
+      <c r="C170" s="8">
         <v>21421112</v>
       </c>
     </row>
@@ -4987,7 +4506,7 @@
       <c r="B190" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="C190" s="10">
+      <c r="C190" s="9">
         <v>21421</v>
       </c>
     </row>
@@ -4998,7 +4517,7 @@
       <c r="B191" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="C191" s="11">
+      <c r="C191" s="10">
         <v>21423</v>
       </c>
     </row>
@@ -5009,7 +4528,7 @@
       <c r="B192" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="C192" s="11">
+      <c r="C192" s="10">
         <v>214211</v>
       </c>
     </row>
@@ -5020,7 +4539,7 @@
       <c r="B193" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="C193" s="11">
+      <c r="C193" s="10">
         <v>2142113</v>
       </c>
     </row>
@@ -5031,7 +4550,7 @@
       <c r="B194" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="C194" s="10">
+      <c r="C194" s="9">
         <v>223223</v>
       </c>
     </row>
@@ -5141,7 +4660,7 @@
       <c r="B204" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="C204" s="11">
+      <c r="C204" s="10">
         <v>21624214</v>
       </c>
     </row>
@@ -5152,7 +4671,7 @@
       <c r="B205" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="C205" s="11">
+      <c r="C205" s="10">
         <v>2162421</v>
       </c>
     </row>
@@ -5163,7 +4682,7 @@
       <c r="B206" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="C206" s="11">
+      <c r="C206" s="10">
         <v>216242</v>
       </c>
     </row>
@@ -5614,7 +5133,7 @@
       <c r="B247" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="C247" s="11">
+      <c r="C247" s="10">
         <v>2233132</v>
       </c>
     </row>
@@ -5669,7 +5188,7 @@
       <c r="B252" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="C252" s="11">
+      <c r="C252" s="10">
         <v>223311335</v>
       </c>
     </row>
@@ -5724,7 +5243,7 @@
       <c r="B257" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="C257" s="11">
+      <c r="C257" s="10">
         <v>223313123</v>
       </c>
     </row>
@@ -5779,7 +5298,7 @@
       <c r="B262" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="C262" s="11">
+      <c r="C262" s="10">
         <v>223311</v>
       </c>
     </row>
@@ -5834,7 +5353,7 @@
       <c r="B267" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="C267" s="11">
+      <c r="C267" s="10">
         <v>2233112</v>
       </c>
     </row>
@@ -5900,7 +5419,7 @@
       <c r="B273" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="C273" s="11">
+      <c r="C273" s="10">
         <v>21624215</v>
       </c>
     </row>
@@ -5966,7 +5485,7 @@
       <c r="B279" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="C279" s="11">
+      <c r="C279" s="10">
         <v>216242144231</v>
       </c>
     </row>
@@ -6032,7 +5551,7 @@
       <c r="B285" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="C285" s="11">
+      <c r="C285" s="10">
         <v>2233121</v>
       </c>
     </row>
@@ -6084,7 +5603,7 @@
       <c r="A290" t="s">
         <v>2</v>
       </c>
-      <c r="B290" s="12" t="s">
+      <c r="B290" s="11" t="s">
         <v>293</v>
       </c>
       <c r="C290" s="2">
@@ -6095,7 +5614,7 @@
       <c r="A291" t="s">
         <v>2</v>
       </c>
-      <c r="B291" s="12" t="s">
+      <c r="B291" s="11" t="s">
         <v>294</v>
       </c>
       <c r="C291" s="2">
@@ -6106,10 +5625,10 @@
       <c r="A292" t="s">
         <v>2</v>
       </c>
-      <c r="B292" s="12" t="s">
+      <c r="B292" s="11" t="s">
         <v>295</v>
       </c>
-      <c r="C292" s="11">
+      <c r="C292" s="10">
         <v>33222</v>
       </c>
     </row>
@@ -6117,7 +5636,7 @@
       <c r="A293" t="s">
         <v>2</v>
       </c>
-      <c r="B293" s="12" t="s">
+      <c r="B293" s="11" t="s">
         <v>296</v>
       </c>
       <c r="C293" s="2">
@@ -6128,7 +5647,7 @@
       <c r="A294" t="s">
         <v>2</v>
       </c>
-      <c r="B294" s="12" t="s">
+      <c r="B294" s="11" t="s">
         <v>297</v>
       </c>
       <c r="C294" s="2">
@@ -6139,7 +5658,7 @@
       <c r="A295" t="s">
         <v>2</v>
       </c>
-      <c r="B295" s="12" t="s">
+      <c r="B295" s="11" t="s">
         <v>298</v>
       </c>
       <c r="C295" s="2">
@@ -6150,7 +5669,7 @@
       <c r="A296" t="s">
         <v>2</v>
       </c>
-      <c r="B296" s="12" t="s">
+      <c r="B296" s="11" t="s">
         <v>299</v>
       </c>
       <c r="C296" s="2">
@@ -6161,7 +5680,7 @@
       <c r="A297" t="s">
         <v>2</v>
       </c>
-      <c r="B297" s="12" t="s">
+      <c r="B297" s="11" t="s">
         <v>300</v>
       </c>
       <c r="C297" s="2">
@@ -6172,10 +5691,10 @@
       <c r="A298" t="s">
         <v>2</v>
       </c>
-      <c r="B298" s="12" t="s">
+      <c r="B298" s="11" t="s">
         <v>301</v>
       </c>
-      <c r="C298" s="11">
+      <c r="C298" s="10">
         <v>33511</v>
       </c>
     </row>
@@ -6183,7 +5702,7 @@
       <c r="A299" t="s">
         <v>2</v>
       </c>
-      <c r="B299" s="12" t="s">
+      <c r="B299" s="11" t="s">
         <v>302</v>
       </c>
       <c r="C299" s="2">
@@ -6194,7 +5713,7 @@
       <c r="A300" t="s">
         <v>2</v>
       </c>
-      <c r="B300" s="12" t="s">
+      <c r="B300" s="11" t="s">
         <v>303</v>
       </c>
       <c r="C300" s="2">
@@ -6205,7 +5724,7 @@
       <c r="A301" t="s">
         <v>2</v>
       </c>
-      <c r="B301" s="12" t="s">
+      <c r="B301" s="11" t="s">
         <v>304</v>
       </c>
       <c r="C301" s="2">
@@ -6216,7 +5735,7 @@
       <c r="A302" t="s">
         <v>2</v>
       </c>
-      <c r="B302" s="12" t="s">
+      <c r="B302" s="11" t="s">
         <v>305</v>
       </c>
       <c r="C302" s="2">
@@ -6227,7 +5746,7 @@
       <c r="A303" t="s">
         <v>2</v>
       </c>
-      <c r="B303" s="12" t="s">
+      <c r="B303" s="11" t="s">
         <v>306</v>
       </c>
       <c r="C303" s="2">
@@ -6238,10 +5757,10 @@
       <c r="A304" t="s">
         <v>2</v>
       </c>
-      <c r="B304" s="12" t="s">
+      <c r="B304" s="11" t="s">
         <v>307</v>
       </c>
-      <c r="C304" s="11">
+      <c r="C304" s="10">
         <v>31431</v>
       </c>
     </row>
@@ -6249,7 +5768,7 @@
       <c r="A305" t="s">
         <v>2</v>
       </c>
-      <c r="B305" s="12" t="s">
+      <c r="B305" s="11" t="s">
         <v>308</v>
       </c>
       <c r="C305" s="2">
@@ -6260,7 +5779,7 @@
       <c r="A306" t="s">
         <v>2</v>
       </c>
-      <c r="B306" s="12" t="s">
+      <c r="B306" s="11" t="s">
         <v>309</v>
       </c>
       <c r="C306" s="2">
@@ -6271,7 +5790,7 @@
       <c r="A307" t="s">
         <v>2</v>
       </c>
-      <c r="B307" s="12" t="s">
+      <c r="B307" s="11" t="s">
         <v>310</v>
       </c>
       <c r="C307" s="2">
@@ -6282,7 +5801,7 @@
       <c r="A308" t="s">
         <v>2</v>
       </c>
-      <c r="B308" s="12" t="s">
+      <c r="B308" s="11" t="s">
         <v>311</v>
       </c>
       <c r="C308" s="2">
@@ -6293,7 +5812,7 @@
       <c r="A309" t="s">
         <v>2</v>
       </c>
-      <c r="B309" s="12" t="s">
+      <c r="B309" s="11" t="s">
         <v>312</v>
       </c>
       <c r="C309" s="2">
@@ -6304,10 +5823,10 @@
       <c r="A310" t="s">
         <v>2</v>
       </c>
-      <c r="B310" s="12" t="s">
+      <c r="B310" s="11" t="s">
         <v>313</v>
       </c>
-      <c r="C310" s="11">
+      <c r="C310" s="10">
         <v>3111121</v>
       </c>
     </row>
@@ -6315,7 +5834,7 @@
       <c r="A311" t="s">
         <v>2</v>
       </c>
-      <c r="B311" s="12" t="s">
+      <c r="B311" s="11" t="s">
         <v>314</v>
       </c>
       <c r="C311" s="2">
@@ -6326,7 +5845,7 @@
       <c r="A312" t="s">
         <v>2</v>
       </c>
-      <c r="B312" s="12" t="s">
+      <c r="B312" s="11" t="s">
         <v>315</v>
       </c>
       <c r="C312" s="2">
@@ -6337,7 +5856,7 @@
       <c r="A313" t="s">
         <v>2</v>
       </c>
-      <c r="B313" s="12" t="s">
+      <c r="B313" s="11" t="s">
         <v>316</v>
       </c>
       <c r="C313" s="2">
@@ -6348,7 +5867,7 @@
       <c r="A314" t="s">
         <v>2</v>
       </c>
-      <c r="B314" s="12" t="s">
+      <c r="B314" s="11" t="s">
         <v>317</v>
       </c>
       <c r="C314" s="2">
@@ -6359,7 +5878,7 @@
       <c r="A315" t="s">
         <v>2</v>
       </c>
-      <c r="B315" s="12" t="s">
+      <c r="B315" s="11" t="s">
         <v>318</v>
       </c>
       <c r="C315" s="2">
@@ -6370,10 +5889,10 @@
       <c r="A316" t="s">
         <v>2</v>
       </c>
-      <c r="B316" s="12" t="s">
+      <c r="B316" s="11" t="s">
         <v>319</v>
       </c>
-      <c r="C316" s="11">
+      <c r="C316" s="10">
         <v>31432314</v>
       </c>
     </row>
@@ -6381,7 +5900,7 @@
       <c r="A317" t="s">
         <v>2</v>
       </c>
-      <c r="B317" s="12" t="s">
+      <c r="B317" s="11" t="s">
         <v>320</v>
       </c>
       <c r="C317" s="2">
@@ -6392,7 +5911,7 @@
       <c r="A318" t="s">
         <v>2</v>
       </c>
-      <c r="B318" s="12" t="s">
+      <c r="B318" s="11" t="s">
         <v>321</v>
       </c>
       <c r="C318" s="2">
@@ -6403,7 +5922,7 @@
       <c r="A319" t="s">
         <v>2</v>
       </c>
-      <c r="B319" s="12" t="s">
+      <c r="B319" s="11" t="s">
         <v>322</v>
       </c>
       <c r="C319" s="2">
@@ -6414,7 +5933,7 @@
       <c r="A320" t="s">
         <v>2</v>
       </c>
-      <c r="B320" s="12" t="s">
+      <c r="B320" s="11" t="s">
         <v>323</v>
       </c>
       <c r="C320" s="2">
@@ -6425,7 +5944,7 @@
       <c r="A321" t="s">
         <v>2</v>
       </c>
-      <c r="B321" s="12" t="s">
+      <c r="B321" s="11" t="s">
         <v>324</v>
       </c>
       <c r="C321" s="2">
@@ -6436,10 +5955,10 @@
       <c r="A322" t="s">
         <v>2</v>
       </c>
-      <c r="B322" s="12" t="s">
+      <c r="B322" s="11" t="s">
         <v>325</v>
       </c>
-      <c r="C322" s="11">
+      <c r="C322" s="10">
         <v>3113</v>
       </c>
     </row>
@@ -6447,7 +5966,7 @@
       <c r="A323" t="s">
         <v>2</v>
       </c>
-      <c r="B323" s="12" t="s">
+      <c r="B323" s="11" t="s">
         <v>326</v>
       </c>
       <c r="C323" s="2">
@@ -6458,7 +5977,7 @@
       <c r="A324" t="s">
         <v>2</v>
       </c>
-      <c r="B324" s="12" t="s">
+      <c r="B324" s="11" t="s">
         <v>327</v>
       </c>
       <c r="C324" s="2">
@@ -6469,7 +5988,7 @@
       <c r="A325" t="s">
         <v>2</v>
       </c>
-      <c r="B325" s="12" t="s">
+      <c r="B325" s="11" t="s">
         <v>328</v>
       </c>
       <c r="C325" s="2">
@@ -6480,7 +5999,7 @@
       <c r="A326" t="s">
         <v>2</v>
       </c>
-      <c r="B326" s="12" t="s">
+      <c r="B326" s="11" t="s">
         <v>329</v>
       </c>
       <c r="C326" s="2">
@@ -6491,7 +6010,7 @@
       <c r="A327" t="s">
         <v>2</v>
       </c>
-      <c r="B327" s="12" t="s">
+      <c r="B327" s="11" t="s">
         <v>330</v>
       </c>
       <c r="C327" s="2">
@@ -6502,10 +6021,10 @@
       <c r="A328" t="s">
         <v>2</v>
       </c>
-      <c r="B328" s="12" t="s">
+      <c r="B328" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="C328" s="11">
+      <c r="C328" s="10">
         <v>311113</v>
       </c>
     </row>
@@ -6513,7 +6032,7 @@
       <c r="A329" t="s">
         <v>2</v>
       </c>
-      <c r="B329" s="12" t="s">
+      <c r="B329" s="11" t="s">
         <v>332</v>
       </c>
       <c r="C329" s="2">
@@ -6524,7 +6043,7 @@
       <c r="A330" t="s">
         <v>2</v>
       </c>
-      <c r="B330" s="12" t="s">
+      <c r="B330" s="11" t="s">
         <v>333</v>
       </c>
       <c r="C330" s="2">
@@ -6535,7 +6054,7 @@
       <c r="A331" t="s">
         <v>2</v>
       </c>
-      <c r="B331" s="12" t="s">
+      <c r="B331" s="11" t="s">
         <v>334</v>
       </c>
       <c r="C331" s="2">
@@ -6546,7 +6065,7 @@
       <c r="A332" t="s">
         <v>2</v>
       </c>
-      <c r="B332" s="12" t="s">
+      <c r="B332" s="11" t="s">
         <v>335</v>
       </c>
       <c r="C332" s="2">
@@ -6557,7 +6076,7 @@
       <c r="A333" t="s">
         <v>2</v>
       </c>
-      <c r="B333" s="12" t="s">
+      <c r="B333" s="11" t="s">
         <v>336</v>
       </c>
       <c r="C333" s="2">
@@ -6568,10 +6087,10 @@
       <c r="A334" t="s">
         <v>2</v>
       </c>
-      <c r="B334" s="12" t="s">
+      <c r="B334" s="11" t="s">
         <v>337</v>
       </c>
-      <c r="C334" s="11">
+      <c r="C334" s="10">
         <v>3131</v>
       </c>
     </row>
@@ -6579,7 +6098,7 @@
       <c r="A335" t="s">
         <v>2</v>
       </c>
-      <c r="B335" s="12" t="s">
+      <c r="B335" s="11" t="s">
         <v>338</v>
       </c>
       <c r="C335" s="2">
@@ -6590,7 +6109,7 @@
       <c r="A336" t="s">
         <v>2</v>
       </c>
-      <c r="B336" s="12" t="s">
+      <c r="B336" s="11" t="s">
         <v>339</v>
       </c>
       <c r="C336" s="2">
@@ -6601,7 +6120,7 @@
       <c r="A337" t="s">
         <v>2</v>
       </c>
-      <c r="B337" s="12" t="s">
+      <c r="B337" s="11" t="s">
         <v>340</v>
       </c>
       <c r="C337" s="2">
@@ -6612,7 +6131,7 @@
       <c r="A338" t="s">
         <v>2</v>
       </c>
-      <c r="B338" s="12" t="s">
+      <c r="B338" s="11" t="s">
         <v>341</v>
       </c>
       <c r="C338" s="2">
@@ -6623,7 +6142,7 @@
       <c r="A339" t="s">
         <v>2</v>
       </c>
-      <c r="B339" s="12" t="s">
+      <c r="B339" s="11" t="s">
         <v>342</v>
       </c>
       <c r="C339" s="2">
@@ -6634,10 +6153,10 @@
       <c r="A340" t="s">
         <v>2</v>
       </c>
-      <c r="B340" s="12" t="s">
+      <c r="B340" s="11" t="s">
         <v>343</v>
       </c>
-      <c r="C340" s="11">
+      <c r="C340" s="10">
         <v>31422</v>
       </c>
     </row>
@@ -6645,7 +6164,7 @@
       <c r="A341" t="s">
         <v>2</v>
       </c>
-      <c r="B341" s="12" t="s">
+      <c r="B341" s="11" t="s">
         <v>344</v>
       </c>
       <c r="C341" s="2">
@@ -6656,7 +6175,7 @@
       <c r="A342" t="s">
         <v>2</v>
       </c>
-      <c r="B342" s="12" t="s">
+      <c r="B342" s="11" t="s">
         <v>345</v>
       </c>
       <c r="C342" s="2">
@@ -6667,7 +6186,7 @@
       <c r="A343" t="s">
         <v>2</v>
       </c>
-      <c r="B343" s="12" t="s">
+      <c r="B343" s="11" t="s">
         <v>346</v>
       </c>
       <c r="C343" s="2">
@@ -6678,7 +6197,7 @@
       <c r="A344" t="s">
         <v>2</v>
       </c>
-      <c r="B344" s="12" t="s">
+      <c r="B344" s="11" t="s">
         <v>347</v>
       </c>
       <c r="C344" s="2">
@@ -6689,7 +6208,7 @@
       <c r="A345" t="s">
         <v>2</v>
       </c>
-      <c r="B345" s="12" t="s">
+      <c r="B345" s="11" t="s">
         <v>348</v>
       </c>
       <c r="C345" s="2">
@@ -6700,10 +6219,10 @@
       <c r="A346" t="s">
         <v>2</v>
       </c>
-      <c r="B346" s="12" t="s">
+      <c r="B346" s="11" t="s">
         <v>349</v>
       </c>
-      <c r="C346" s="11">
+      <c r="C346" s="10">
         <v>336</v>
       </c>
     </row>
@@ -6711,7 +6230,7 @@
       <c r="A347" t="s">
         <v>2</v>
       </c>
-      <c r="B347" s="12" t="s">
+      <c r="B347" s="11" t="s">
         <v>350</v>
       </c>
       <c r="C347" s="2">
@@ -6722,7 +6241,7 @@
       <c r="A348" t="s">
         <v>2</v>
       </c>
-      <c r="B348" s="12" t="s">
+      <c r="B348" s="11" t="s">
         <v>351</v>
       </c>
       <c r="C348" s="2">
@@ -6733,7 +6252,7 @@
       <c r="A349" t="s">
         <v>2</v>
       </c>
-      <c r="B349" s="12" t="s">
+      <c r="B349" s="11" t="s">
         <v>352</v>
       </c>
       <c r="C349" s="2">
@@ -6744,7 +6263,7 @@
       <c r="A350" t="s">
         <v>2</v>
       </c>
-      <c r="B350" s="12" t="s">
+      <c r="B350" s="11" t="s">
         <v>353</v>
       </c>
       <c r="C350" s="2">
@@ -6755,7 +6274,7 @@
       <c r="A351" t="s">
         <v>2</v>
       </c>
-      <c r="B351" s="12" t="s">
+      <c r="B351" s="11" t="s">
         <v>354</v>
       </c>
       <c r="C351" s="2">
@@ -6766,10 +6285,10 @@
       <c r="A352" t="s">
         <v>2</v>
       </c>
-      <c r="B352" s="12" t="s">
+      <c r="B352" s="11" t="s">
         <v>355</v>
       </c>
-      <c r="C352" s="11">
+      <c r="C352" s="10">
         <v>321</v>
       </c>
     </row>
@@ -6777,10 +6296,10 @@
       <c r="A353" t="s">
         <v>2</v>
       </c>
-      <c r="B353" s="12" t="s">
+      <c r="B353" s="11" t="s">
         <v>356</v>
       </c>
-      <c r="C353" s="11">
+      <c r="C353" s="10">
         <v>351</v>
       </c>
     </row>
@@ -6788,10 +6307,10 @@
       <c r="A354" t="s">
         <v>2</v>
       </c>
-      <c r="B354" s="12" t="s">
+      <c r="B354" s="11" t="s">
         <v>357</v>
       </c>
-      <c r="C354" s="11">
+      <c r="C354" s="10">
         <v>31411</v>
       </c>
     </row>
@@ -6799,10 +6318,10 @@
       <c r="A355" t="s">
         <v>2</v>
       </c>
-      <c r="B355" s="12" t="s">
+      <c r="B355" s="11" t="s">
         <v>358</v>
       </c>
-      <c r="C355" s="11">
+      <c r="C355" s="10">
         <v>32</v>
       </c>
     </row>
@@ -6810,10 +6329,10 @@
       <c r="A356" t="s">
         <v>2</v>
       </c>
-      <c r="B356" s="12" t="s">
+      <c r="B356" s="11" t="s">
         <v>359</v>
       </c>
-      <c r="C356" s="11">
+      <c r="C356" s="10">
         <v>33</v>
       </c>
     </row>
@@ -6821,10 +6340,10 @@
       <c r="A357" t="s">
         <v>2</v>
       </c>
-      <c r="B357" s="12" t="s">
+      <c r="B357" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="C357" s="11">
+      <c r="C357" s="10">
         <v>31</v>
       </c>
     </row>
@@ -6832,10 +6351,10 @@
       <c r="A358" t="s">
         <v>2</v>
       </c>
-      <c r="B358" s="12" t="s">
+      <c r="B358" s="11" t="s">
         <v>361</v>
       </c>
-      <c r="C358" s="11">
+      <c r="C358" s="10">
         <v>3143234</v>
       </c>
     </row>
@@ -6843,10 +6362,10 @@
       <c r="A359" t="s">
         <v>2</v>
       </c>
-      <c r="B359" s="12" t="s">
+      <c r="B359" s="11" t="s">
         <v>362</v>
       </c>
-      <c r="C359" s="11">
+      <c r="C359" s="10">
         <v>33223</v>
       </c>
     </row>
@@ -6854,10 +6373,10 @@
       <c r="A360" t="s">
         <v>2</v>
       </c>
-      <c r="B360" s="12" t="s">
+      <c r="B360" s="11" t="s">
         <v>363</v>
       </c>
-      <c r="C360" s="11">
+      <c r="C360" s="10">
         <v>314321</v>
       </c>
     </row>
@@ -6865,10 +6384,10 @@
       <c r="A361" t="s">
         <v>2</v>
       </c>
-      <c r="B361" s="12" t="s">
+      <c r="B361" s="11" t="s">
         <v>364</v>
       </c>
-      <c r="C361" s="11">
+      <c r="C361" s="10">
         <v>31432131</v>
       </c>
     </row>
@@ -6876,10 +6395,10 @@
       <c r="A362" t="s">
         <v>2</v>
       </c>
-      <c r="B362" s="12" t="s">
+      <c r="B362" s="11" t="s">
         <v>365</v>
       </c>
-      <c r="C362" s="11">
+      <c r="C362" s="10">
         <v>314311</v>
       </c>
     </row>
@@ -6887,10 +6406,10 @@
       <c r="A363" t="s">
         <v>2</v>
       </c>
-      <c r="B363" s="12" t="s">
+      <c r="B363" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="C363" s="11">
+      <c r="C363" s="10">
         <v>314323</v>
       </c>
     </row>
@@ -6898,10 +6417,10 @@
       <c r="A364" t="s">
         <v>2</v>
       </c>
-      <c r="B364" s="12" t="s">
+      <c r="B364" s="11" t="s">
         <v>367</v>
       </c>
-      <c r="C364" s="11">
+      <c r="C364" s="10">
         <v>314325312</v>
       </c>
     </row>
@@ -6909,10 +6428,10 @@
       <c r="A365" t="s">
         <v>2</v>
       </c>
-      <c r="B365" s="12" t="s">
+      <c r="B365" s="11" t="s">
         <v>368</v>
       </c>
-      <c r="C365" s="11">
+      <c r="C365" s="10">
         <v>314325313</v>
       </c>
     </row>
@@ -6920,10 +6439,10 @@
       <c r="A366" t="s">
         <v>2</v>
       </c>
-      <c r="B366" s="12" t="s">
+      <c r="B366" s="11" t="s">
         <v>369</v>
       </c>
-      <c r="C366" s="11">
+      <c r="C366" s="10">
         <v>3143253123</v>
       </c>
     </row>
@@ -6931,10 +6450,10 @@
       <c r="A367" t="s">
         <v>2</v>
       </c>
-      <c r="B367" s="12" t="s">
+      <c r="B367" s="11" t="s">
         <v>370</v>
       </c>
-      <c r="C367" s="11">
+      <c r="C367" s="10">
         <v>31432315</v>
       </c>
     </row>
@@ -6942,10 +6461,10 @@
       <c r="A368" t="s">
         <v>2</v>
       </c>
-      <c r="B368" s="12" t="s">
+      <c r="B368" s="11" t="s">
         <v>371</v>
       </c>
-      <c r="C368" s="11">
+      <c r="C368" s="10">
         <v>3143252</v>
       </c>
     </row>
@@ -6953,10 +6472,10 @@
       <c r="A369" t="s">
         <v>2</v>
       </c>
-      <c r="B369" s="12" t="s">
+      <c r="B369" s="11" t="s">
         <v>372</v>
       </c>
-      <c r="C369" s="11">
+      <c r="C369" s="10">
         <v>3143251</v>
       </c>
     </row>
@@ -6964,10 +6483,10 @@
       <c r="A370" t="s">
         <v>2</v>
       </c>
-      <c r="B370" s="12" t="s">
+      <c r="B370" s="11" t="s">
         <v>373</v>
       </c>
-      <c r="C370" s="11">
+      <c r="C370" s="10">
         <v>31432311</v>
       </c>
     </row>
@@ -6975,10 +6494,10 @@
       <c r="A371" t="s">
         <v>2</v>
       </c>
-      <c r="B371" s="12" t="s">
+      <c r="B371" s="11" t="s">
         <v>374</v>
       </c>
-      <c r="C371" s="11">
+      <c r="C371" s="10">
         <v>314323132</v>
       </c>
     </row>
@@ -6986,10 +6505,10 @@
       <c r="A372" t="s">
         <v>2</v>
       </c>
-      <c r="B372" s="12" t="s">
+      <c r="B372" s="11" t="s">
         <v>375</v>
       </c>
-      <c r="C372" s="11">
+      <c r="C372" s="10">
         <v>314321313</v>
       </c>
     </row>
@@ -6997,10 +6516,10 @@
       <c r="A373" t="s">
         <v>2</v>
       </c>
-      <c r="B373" s="12" t="s">
+      <c r="B373" s="11" t="s">
         <v>376</v>
       </c>
-      <c r="C373" s="11">
+      <c r="C373" s="10">
         <v>314325311</v>
       </c>
     </row>
@@ -7008,10 +6527,10 @@
       <c r="A374" t="s">
         <v>2</v>
       </c>
-      <c r="B374" s="12" t="s">
+      <c r="B374" s="11" t="s">
         <v>377</v>
       </c>
-      <c r="C374" s="11">
+      <c r="C374" s="10">
         <v>3322</v>
       </c>
     </row>
@@ -7019,10 +6538,10 @@
       <c r="A375" t="s">
         <v>2</v>
       </c>
-      <c r="B375" s="12" t="s">
+      <c r="B375" s="11" t="s">
         <v>378</v>
       </c>
-      <c r="C375" s="11">
+      <c r="C375" s="10">
         <v>34</v>
       </c>
     </row>
@@ -7030,10 +6549,10 @@
       <c r="A376" t="s">
         <v>2</v>
       </c>
-      <c r="B376" s="12" t="s">
+      <c r="B376" s="11" t="s">
         <v>379</v>
       </c>
-      <c r="C376" s="13">
+      <c r="C376" s="12">
         <v>31213</v>
       </c>
     </row>
@@ -7041,10 +6560,10 @@
       <c r="A377" t="s">
         <v>2</v>
       </c>
-      <c r="B377" s="12" t="s">
+      <c r="B377" s="11" t="s">
         <v>380</v>
       </c>
-      <c r="C377" s="13">
+      <c r="C377" s="12">
         <v>311</v>
       </c>
     </row>
@@ -7052,10 +6571,10 @@
       <c r="A378" t="s">
         <v>2</v>
       </c>
-      <c r="B378" s="12" t="s">
+      <c r="B378" s="11" t="s">
         <v>381</v>
       </c>
-      <c r="C378" s="13">
+      <c r="C378" s="12">
         <v>332222</v>
       </c>
     </row>
@@ -7063,10 +6582,10 @@
       <c r="A379" t="s">
         <v>2</v>
       </c>
-      <c r="B379" s="12" t="s">
+      <c r="B379" s="11" t="s">
         <v>382</v>
       </c>
-      <c r="C379" s="13">
+      <c r="C379" s="12">
         <v>314323135</v>
       </c>
     </row>
@@ -7074,10 +6593,10 @@
       <c r="A380" t="s">
         <v>2</v>
       </c>
-      <c r="B380" s="12" t="s">
+      <c r="B380" s="11" t="s">
         <v>383</v>
       </c>
-      <c r="C380" s="13">
+      <c r="C380" s="12">
         <v>314323134</v>
       </c>
     </row>
@@ -7085,10 +6604,10 @@
       <c r="A381" t="s">
         <v>2</v>
       </c>
-      <c r="B381" s="12" t="s">
+      <c r="B381" s="11" t="s">
         <v>384</v>
       </c>
-      <c r="C381" s="13">
+      <c r="C381" s="12">
         <v>31432313</v>
       </c>
     </row>
@@ -7096,10 +6615,10 @@
       <c r="A382" t="s">
         <v>2</v>
       </c>
-      <c r="B382" s="12" t="s">
+      <c r="B382" s="11" t="s">
         <v>385</v>
       </c>
-      <c r="C382" s="13">
+      <c r="C382" s="12">
         <v>3363</v>
       </c>
     </row>
@@ -7107,10 +6626,10 @@
       <c r="A383" t="s">
         <v>2</v>
       </c>
-      <c r="B383" s="12" t="s">
+      <c r="B383" s="11" t="s">
         <v>386</v>
       </c>
-      <c r="C383" s="13">
+      <c r="C383" s="12">
         <v>3111134</v>
       </c>
     </row>
@@ -7118,10 +6637,10 @@
       <c r="A384" t="s">
         <v>2</v>
       </c>
-      <c r="B384" s="12" t="s">
+      <c r="B384" s="11" t="s">
         <v>387</v>
       </c>
-      <c r="C384" s="13">
+      <c r="C384" s="12">
         <v>31113</v>
       </c>
     </row>
@@ -7129,10 +6648,10 @@
       <c r="A385" t="s">
         <v>2</v>
       </c>
-      <c r="B385" s="12" t="s">
+      <c r="B385" s="11" t="s">
         <v>388</v>
       </c>
-      <c r="C385" s="13">
+      <c r="C385" s="12">
         <v>311111</v>
       </c>
     </row>
@@ -7140,10 +6659,10 @@
       <c r="A386" t="s">
         <v>2</v>
       </c>
-      <c r="B386" s="12" t="s">
+      <c r="B386" s="11" t="s">
         <v>389</v>
       </c>
-      <c r="C386" s="13">
+      <c r="C386" s="12">
         <v>31111</v>
       </c>
     </row>
@@ -7151,10 +6670,10 @@
       <c r="A387" t="s">
         <v>2</v>
       </c>
-      <c r="B387" s="12" t="s">
+      <c r="B387" s="11" t="s">
         <v>390</v>
       </c>
-      <c r="C387" s="13">
+      <c r="C387" s="12">
         <v>332221</v>
       </c>
     </row>
@@ -7162,10 +6681,10 @@
       <c r="A388" t="s">
         <v>2</v>
       </c>
-      <c r="B388" s="12" t="s">
+      <c r="B388" s="11" t="s">
         <v>391</v>
       </c>
-      <c r="C388" s="13">
+      <c r="C388" s="12">
         <v>31432531</v>
       </c>
     </row>
@@ -7173,10 +6692,10 @@
       <c r="A389" t="s">
         <v>2</v>
       </c>
-      <c r="B389" s="12" t="s">
+      <c r="B389" s="11" t="s">
         <v>392</v>
       </c>
-      <c r="C389" s="13">
+      <c r="C389" s="12">
         <v>3143253</v>
       </c>
     </row>
@@ -7184,10 +6703,10 @@
       <c r="A390" t="s">
         <v>2</v>
       </c>
-      <c r="B390" s="12" t="s">
+      <c r="B390" s="11" t="s">
         <v>393</v>
       </c>
-      <c r="C390" s="13">
+      <c r="C390" s="12">
         <v>314325</v>
       </c>
     </row>
@@ -7195,10 +6714,10 @@
       <c r="A391" t="s">
         <v>2</v>
       </c>
-      <c r="B391" s="12" t="s">
+      <c r="B391" s="11" t="s">
         <v>394</v>
       </c>
-      <c r="C391" s="13">
+      <c r="C391" s="12">
         <v>314322</v>
       </c>
     </row>
@@ -7206,10 +6725,10 @@
       <c r="A392" t="s">
         <v>2</v>
       </c>
-      <c r="B392" s="12" t="s">
+      <c r="B392" s="11" t="s">
         <v>395</v>
       </c>
-      <c r="C392" s="13">
+      <c r="C392" s="12">
         <v>314332</v>
       </c>
     </row>
@@ -7217,10 +6736,10 @@
       <c r="A393" t="s">
         <v>2</v>
       </c>
-      <c r="B393" s="12" t="s">
+      <c r="B393" s="11" t="s">
         <v>396</v>
       </c>
-      <c r="C393" s="13">
+      <c r="C393" s="12">
         <v>3143334</v>
       </c>
     </row>
@@ -7228,10 +6747,10 @@
       <c r="A394" t="s">
         <v>2</v>
       </c>
-      <c r="B394" s="12" t="s">
+      <c r="B394" s="11" t="s">
         <v>397</v>
       </c>
-      <c r="C394" s="13">
+      <c r="C394" s="12">
         <v>3143333</v>
       </c>
     </row>
@@ -7239,10 +6758,10 @@
       <c r="A395" t="s">
         <v>2</v>
       </c>
-      <c r="B395" s="12" t="s">
+      <c r="B395" s="11" t="s">
         <v>398</v>
       </c>
-      <c r="C395" s="13">
+      <c r="C395" s="12">
         <v>3143331</v>
       </c>
     </row>
@@ -7250,10 +6769,10 @@
       <c r="A396" t="s">
         <v>2</v>
       </c>
-      <c r="B396" s="12" t="s">
+      <c r="B396" s="11" t="s">
         <v>399</v>
       </c>
-      <c r="C396" s="13">
+      <c r="C396" s="12">
         <v>314333</v>
       </c>
     </row>
@@ -7261,10 +6780,10 @@
       <c r="A397" t="s">
         <v>2</v>
       </c>
-      <c r="B397" s="12" t="s">
+      <c r="B397" s="11" t="s">
         <v>400</v>
       </c>
-      <c r="C397" s="13">
+      <c r="C397" s="12">
         <v>41</v>
       </c>
     </row>
@@ -7272,10 +6791,10 @@
       <c r="A398" t="s">
         <v>2</v>
       </c>
-      <c r="B398" s="12" t="s">
+      <c r="B398" s="11" t="s">
         <v>401</v>
       </c>
-      <c r="C398" s="13">
+      <c r="C398" s="12">
         <v>44</v>
       </c>
     </row>
@@ -7283,10 +6802,10 @@
       <c r="A399" t="s">
         <v>2</v>
       </c>
-      <c r="B399" s="12" t="s">
+      <c r="B399" s="11" t="s">
         <v>402</v>
       </c>
-      <c r="C399" s="13">
+      <c r="C399" s="12">
         <v>4211313</v>
       </c>
     </row>
@@ -7294,10 +6813,10 @@
       <c r="A400" t="s">
         <v>2</v>
       </c>
-      <c r="B400" s="12" t="s">
+      <c r="B400" s="11" t="s">
         <v>403</v>
       </c>
-      <c r="C400" s="13">
+      <c r="C400" s="12">
         <v>421131</v>
       </c>
     </row>
@@ -7305,10 +6824,10 @@
       <c r="A401" t="s">
         <v>2</v>
       </c>
-      <c r="B401" s="12" t="s">
+      <c r="B401" s="11" t="s">
         <v>404</v>
       </c>
-      <c r="C401" s="13">
+      <c r="C401" s="12">
         <v>45</v>
       </c>
     </row>
@@ -7316,10 +6835,10 @@
       <c r="A402" t="s">
         <v>2</v>
       </c>
-      <c r="B402" s="12" t="s">
+      <c r="B402" s="11" t="s">
         <v>405</v>
       </c>
-      <c r="C402" s="13">
+      <c r="C402" s="12">
         <v>42113</v>
       </c>
     </row>
@@ -7327,10 +6846,10 @@
       <c r="A403" t="s">
         <v>2</v>
       </c>
-      <c r="B403" s="12" t="s">
+      <c r="B403" s="11" t="s">
         <v>406</v>
       </c>
-      <c r="C403" s="13">
+      <c r="C403" s="12">
         <v>4212</v>
       </c>
     </row>
@@ -7338,10 +6857,10 @@
       <c r="A404" t="s">
         <v>2</v>
       </c>
-      <c r="B404" s="12" t="s">
+      <c r="B404" s="11" t="s">
         <v>407</v>
       </c>
-      <c r="C404" s="13">
+      <c r="C404" s="12">
         <v>4252</v>
       </c>
     </row>
@@ -7349,10 +6868,10 @@
       <c r="A405" t="s">
         <v>2</v>
       </c>
-      <c r="B405" s="12" t="s">
+      <c r="B405" s="11" t="s">
         <v>408</v>
       </c>
-      <c r="C405" s="13">
+      <c r="C405" s="12">
         <v>42531</v>
       </c>
     </row>
@@ -7360,10 +6879,10 @@
       <c r="A406" t="s">
         <v>2</v>
       </c>
-      <c r="B406" s="12" t="s">
+      <c r="B406" s="11" t="s">
         <v>409</v>
       </c>
-      <c r="C406" s="13">
+      <c r="C406" s="12">
         <v>4253</v>
       </c>
     </row>
@@ -7371,10 +6890,10 @@
       <c r="A407" t="s">
         <v>2</v>
       </c>
-      <c r="B407" s="12" t="s">
+      <c r="B407" s="11" t="s">
         <v>410</v>
       </c>
-      <c r="C407" s="13">
+      <c r="C407" s="12">
         <v>4251</v>
       </c>
     </row>
@@ -7382,10 +6901,10 @@
       <c r="A408" t="s">
         <v>2</v>
       </c>
-      <c r="B408" s="12" t="s">
+      <c r="B408" s="11" t="s">
         <v>411</v>
       </c>
-      <c r="C408" s="13">
+      <c r="C408" s="12">
         <v>4143</v>
       </c>
     </row>
@@ -7393,10 +6912,10 @@
       <c r="A409" t="s">
         <v>2</v>
       </c>
-      <c r="B409" s="12" t="s">
+      <c r="B409" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="C409" s="13">
+      <c r="C409" s="12">
         <v>4141</v>
       </c>
     </row>
@@ -7404,10 +6923,10 @@
       <c r="A410" t="s">
         <v>2</v>
       </c>
-      <c r="B410" s="12" t="s">
+      <c r="B410" s="11" t="s">
         <v>413</v>
       </c>
-      <c r="C410" s="13">
+      <c r="C410" s="12">
         <v>413</v>
       </c>
     </row>
@@ -7415,10 +6934,10 @@
       <c r="A411" t="s">
         <v>2</v>
       </c>
-      <c r="B411" s="12" t="s">
+      <c r="B411" s="11" t="s">
         <v>414</v>
       </c>
-      <c r="C411" s="13">
+      <c r="C411" s="12">
         <v>412</v>
       </c>
     </row>
@@ -7426,10 +6945,10 @@
       <c r="A412" t="s">
         <v>2</v>
       </c>
-      <c r="B412" s="12" t="s">
+      <c r="B412" s="11" t="s">
         <v>415</v>
       </c>
-      <c r="C412" s="13">
+      <c r="C412" s="12">
         <v>4321</v>
       </c>
     </row>
@@ -7437,10 +6956,10 @@
       <c r="A413" t="s">
         <v>2</v>
       </c>
-      <c r="B413" s="12" t="s">
+      <c r="B413" s="11" t="s">
         <v>416</v>
       </c>
-      <c r="C413" s="13">
+      <c r="C413" s="12">
         <v>42221</v>
       </c>
     </row>
@@ -7448,10 +6967,10 @@
       <c r="A414" t="s">
         <v>2</v>
       </c>
-      <c r="B414" s="12" t="s">
+      <c r="B414" s="11" t="s">
         <v>417</v>
       </c>
-      <c r="C414" s="13">
+      <c r="C414" s="12">
         <v>414</v>
       </c>
     </row>
@@ -7459,10 +6978,10 @@
       <c r="A415" t="s">
         <v>2</v>
       </c>
-      <c r="B415" s="12" t="s">
+      <c r="B415" s="11" t="s">
         <v>418</v>
       </c>
-      <c r="C415" s="13">
+      <c r="C415" s="12">
         <v>432</v>
       </c>
     </row>
@@ -7470,10 +6989,10 @@
       <c r="A416" t="s">
         <v>2</v>
       </c>
-      <c r="B416" s="12" t="s">
+      <c r="B416" s="11" t="s">
         <v>419</v>
       </c>
-      <c r="C416" s="13">
+      <c r="C416" s="12">
         <v>4142</v>
       </c>
     </row>
@@ -7481,10 +7000,10 @@
       <c r="A417" t="s">
         <v>2</v>
       </c>
-      <c r="B417" s="12" t="s">
+      <c r="B417" s="11" t="s">
         <v>420</v>
       </c>
-      <c r="C417" s="13">
+      <c r="C417" s="12">
         <v>4222</v>
       </c>
     </row>
@@ -7492,10 +7011,10 @@
       <c r="A418" t="s">
         <v>2</v>
       </c>
-      <c r="B418" s="12" t="s">
+      <c r="B418" s="11" t="s">
         <v>421</v>
       </c>
-      <c r="C418" s="13">
+      <c r="C418" s="12">
         <v>422</v>
       </c>
     </row>
@@ -7503,10 +7022,10 @@
       <c r="A419" t="s">
         <v>2</v>
       </c>
-      <c r="B419" s="12" t="s">
+      <c r="B419" s="11" t="s">
         <v>422</v>
       </c>
-      <c r="C419" s="13">
+      <c r="C419" s="12">
         <v>42111</v>
       </c>
     </row>
@@ -7514,10 +7033,10 @@
       <c r="A420" t="s">
         <v>2</v>
       </c>
-      <c r="B420" s="12" t="s">
+      <c r="B420" s="11" t="s">
         <v>423</v>
       </c>
-      <c r="C420" s="13">
+      <c r="C420" s="12">
         <v>425</v>
       </c>
     </row>
@@ -7525,10 +7044,10 @@
       <c r="A421" t="s">
         <v>2</v>
       </c>
-      <c r="B421" s="12" t="s">
+      <c r="B421" s="11" t="s">
         <v>424</v>
       </c>
-      <c r="C421" s="13">
+      <c r="C421" s="12">
         <v>4211</v>
       </c>
     </row>
@@ -7536,10 +7055,10 @@
       <c r="A422" t="s">
         <v>2</v>
       </c>
-      <c r="B422" s="12" t="s">
+      <c r="B422" s="11" t="s">
         <v>425</v>
       </c>
-      <c r="C422" s="13">
+      <c r="C422" s="12">
         <v>42</v>
       </c>
     </row>
@@ -7547,10 +7066,10 @@
       <c r="A423" t="s">
         <v>2</v>
       </c>
-      <c r="B423" s="12" t="s">
+      <c r="B423" s="11" t="s">
         <v>426</v>
       </c>
-      <c r="C423" s="13">
+      <c r="C423" s="12">
         <v>43</v>
       </c>
     </row>
@@ -7558,10 +7077,10 @@
       <c r="A424" t="s">
         <v>2</v>
       </c>
-      <c r="B424" s="12" t="s">
+      <c r="B424" s="11" t="s">
         <v>427</v>
       </c>
-      <c r="C424" s="13">
+      <c r="C424" s="12">
         <v>46</v>
       </c>
     </row>
@@ -7569,10 +7088,10 @@
       <c r="A425" t="s">
         <v>2</v>
       </c>
-      <c r="B425" s="12" t="s">
+      <c r="B425" s="11" t="s">
         <v>428</v>
       </c>
-      <c r="C425" s="13">
+      <c r="C425" s="12">
         <v>421</v>
       </c>
     </row>
@@ -7580,10 +7099,10 @@
       <c r="A426" t="s">
         <v>2</v>
       </c>
-      <c r="B426" s="12" t="s">
+      <c r="B426" s="11" t="s">
         <v>429</v>
       </c>
-      <c r="C426" s="13">
+      <c r="C426" s="12">
         <v>422214</v>
       </c>
     </row>
@@ -7591,10 +7110,10 @@
       <c r="A427" t="s">
         <v>2</v>
       </c>
-      <c r="B427" s="12" t="s">
+      <c r="B427" s="11" t="s">
         <v>430</v>
       </c>
-      <c r="C427" s="13">
+      <c r="C427" s="12">
         <v>42223</v>
       </c>
     </row>
@@ -7602,10 +7121,10 @@
       <c r="A428" t="s">
         <v>2</v>
       </c>
-      <c r="B428" s="12" t="s">
+      <c r="B428" s="11" t="s">
         <v>431</v>
       </c>
-      <c r="C428" s="13">
+      <c r="C428" s="12">
         <v>422212</v>
       </c>
     </row>
@@ -7613,10 +7132,10 @@
       <c r="A429" t="s">
         <v>2</v>
       </c>
-      <c r="B429" s="12" t="s">
+      <c r="B429" s="11" t="s">
         <v>432</v>
       </c>
-      <c r="C429" s="13">
+      <c r="C429" s="12">
         <v>42224</v>
       </c>
     </row>
@@ -7624,10 +7143,10 @@
       <c r="A430" t="s">
         <v>2</v>
       </c>
-      <c r="B430" s="12" t="s">
+      <c r="B430" s="11" t="s">
         <v>433</v>
       </c>
-      <c r="C430" s="13">
+      <c r="C430" s="12">
         <v>422213</v>
       </c>
     </row>
@@ -7635,10 +7154,10 @@
       <c r="A431" t="s">
         <v>2</v>
       </c>
-      <c r="B431" s="12" t="s">
+      <c r="B431" s="11" t="s">
         <v>434</v>
       </c>
-      <c r="C431" s="13">
+      <c r="C431" s="12">
         <v>422211</v>
       </c>
     </row>
@@ -7646,10 +7165,10 @@
       <c r="A432" t="s">
         <v>2</v>
       </c>
-      <c r="B432" s="12" t="s">
+      <c r="B432" s="11" t="s">
         <v>435</v>
       </c>
-      <c r="C432" s="13">
+      <c r="C432" s="12">
         <v>42222</v>
       </c>
     </row>
@@ -7657,10 +7176,10 @@
       <c r="A433" t="s">
         <v>2</v>
       </c>
-      <c r="B433" s="12" t="s">
+      <c r="B433" s="11" t="s">
         <v>436</v>
       </c>
-      <c r="C433" s="13">
+      <c r="C433" s="12">
         <v>4222134</v>
       </c>
     </row>
@@ -7668,10 +7187,10 @@
       <c r="A434" t="s">
         <v>2</v>
       </c>
-      <c r="B434" s="12" t="s">
+      <c r="B434" s="11" t="s">
         <v>437</v>
       </c>
-      <c r="C434" s="13">
+      <c r="C434" s="12">
         <v>4222131</v>
       </c>
     </row>
@@ -7679,10 +7198,10 @@
       <c r="A435" t="s">
         <v>2</v>
       </c>
-      <c r="B435" s="12" t="s">
+      <c r="B435" s="11" t="s">
         <v>438</v>
       </c>
-      <c r="C435" s="13">
+      <c r="C435" s="12">
         <v>4222133</v>
       </c>
     </row>
@@ -7690,10 +7209,10 @@
       <c r="A436" t="s">
         <v>2</v>
       </c>
-      <c r="B436" s="12" t="s">
+      <c r="B436" s="11" t="s">
         <v>439</v>
       </c>
-      <c r="C436" s="13">
+      <c r="C436" s="12">
         <v>1132231</v>
       </c>
     </row>
@@ -7701,10 +7220,10 @@
       <c r="A437" t="s">
         <v>2</v>
       </c>
-      <c r="B437" s="12" t="s">
+      <c r="B437" s="11" t="s">
         <v>440</v>
       </c>
-      <c r="C437" s="13">
+      <c r="C437" s="12">
         <v>314</v>
       </c>
     </row>
@@ -7712,28 +7231,28 @@
       <c r="A438" t="s">
         <v>2</v>
       </c>
-      <c r="B438" s="12" t="s">
+      <c r="B438" s="11" t="s">
         <v>441</v>
       </c>
-      <c r="C438" s="13">
+      <c r="C438" s="12">
         <v>332</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B439">
-    <cfRule type="cellIs" dxfId="15" priority="4" operator="notBetween">
+    <cfRule type="cellIs" dxfId="13" priority="4" operator="notBetween">
       <formula>1</formula>
       <formula>500</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C438">
-    <cfRule type="expression" dxfId="14" priority="18">
+    <cfRule type="expression" dxfId="12" priority="18">
       <formula>(COUNTIF(#REF!,$C6))&lt;1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="19">
+    <cfRule type="expression" dxfId="11" priority="19">
       <formula>#REF!&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="notContainsBlanks" dxfId="12" priority="20">
+    <cfRule type="notContainsBlanks" dxfId="10" priority="20">
       <formula>LEN(TRIM(C6))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7761,268 +7280,268 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="86" t="s">
+      <c r="C2" s="51" t="s">
         <v>442</v>
       </c>
-      <c r="D2" s="83"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="87">
+      <c r="D2" s="52"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="53">
         <f ca="1">TODAY()</f>
-        <v>45672</v>
-      </c>
-      <c r="G2" s="85"/>
-      <c r="H2" s="84"/>
+        <v>46069</v>
+      </c>
+      <c r="G2" s="54"/>
+      <c r="H2" s="55"/>
     </row>
     <row r="3" spans="3:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
     </row>
     <row r="4" spans="3:8" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="3:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
     </row>
     <row r="6" spans="3:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="15" t="s">
         <v>443</v>
       </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="88" t="s">
+      <c r="D6" s="16"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="56" t="s">
         <v>444</v>
       </c>
-      <c r="G6" s="89"/>
-      <c r="H6" s="90"/>
+      <c r="G6" s="57"/>
+      <c r="H6" s="58"/>
     </row>
     <row r="7" spans="3:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="18"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="92"/>
-      <c r="H7" s="93"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="59"/>
+      <c r="G7" s="60"/>
+      <c r="H7" s="61"/>
     </row>
     <row r="8" spans="3:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="15" t="s">
         <v>445</v>
       </c>
       <c r="D8" s="1">
         <v>2</v>
       </c>
-      <c r="E8" s="14"/>
-      <c r="F8" s="94"/>
-      <c r="G8" s="95"/>
-      <c r="H8" s="96"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="62"/>
+      <c r="G8" s="63"/>
+      <c r="H8" s="64"/>
     </row>
     <row r="9" spans="3:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="19"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="3:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C10" s="16"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
     </row>
     <row r="11" spans="3:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C11" s="25"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
     </row>
     <row r="12" spans="3:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="27" t="s">
         <v>446</v>
       </c>
-      <c r="D12" s="29" t="e">
+      <c r="D12" s="28" t="e">
         <f>IF(D8&lt;&gt;0,(VLOOKUP(D8,CTF!$B$2:$C$193,2,FALSE)),D6)</f>
         <v>#N/A</v>
       </c>
-      <c r="E12" s="30"/>
-      <c r="F12" s="31" t="e">
+      <c r="E12" s="29"/>
+      <c r="F12" s="30" t="e">
         <f>IF(COUNTIF(CTF!#REF!,D12)=1,"VALID","NOT VALID")</f>
         <v>#REF!</v>
       </c>
-      <c r="G12" s="30"/>
-      <c r="H12" s="32"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="31"/>
     </row>
     <row r="13" spans="3:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="34"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
     </row>
     <row r="14" spans="3:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="27" t="s">
         <v>447</v>
       </c>
-      <c r="D14" s="37" t="e">
+      <c r="D14" s="36" t="e">
         <f t="array" ref="D14">INDEX(CTF!#REF!,MATCH(TRUE,MMULT(--(CTF!#REF!=D12),TRANSPOSE(COLUMN(CTF!#REF!)^0))&gt;0,0))</f>
         <v>#REF!</v>
       </c>
-      <c r="E14" s="30"/>
-      <c r="F14" s="38" t="e">
+      <c r="E14" s="29"/>
+      <c r="F14" s="37" t="e">
         <f ca="1">IF(D14&lt;F2,"EXPIRED","VALID")</f>
         <v>#REF!</v>
       </c>
-      <c r="G14" s="30"/>
-      <c r="H14" s="32"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="31"/>
     </row>
     <row r="18" spans="3:10" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C18" s="39" t="s">
+      <c r="C18" s="38" t="s">
         <v>448</v>
       </c>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="14"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="35"/>
+      <c r="J18" s="13"/>
     </row>
     <row r="19" spans="3:10" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="39"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="35"/>
-      <c r="H19" s="35"/>
-      <c r="I19" s="36"/>
-      <c r="J19" s="14"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="35"/>
+      <c r="J19" s="13"/>
     </row>
     <row r="20" spans="3:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C20" s="35" t="s">
+      <c r="C20" s="34" t="s">
         <v>449</v>
       </c>
-      <c r="D20" s="40">
+      <c r="D20" s="39">
         <v>6</v>
       </c>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35"/>
-      <c r="G20" s="35"/>
-      <c r="H20" s="35"/>
-      <c r="I20" s="36"/>
-      <c r="J20" s="14"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="34"/>
+      <c r="I20" s="35"/>
+      <c r="J20" s="13"/>
     </row>
     <row r="21" spans="3:10" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="35"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35"/>
-      <c r="G21" s="35"/>
-      <c r="H21" s="35"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="14" t="s">
+      <c r="C21" s="34"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="35"/>
+      <c r="J21" s="13" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="3:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="29" t="s">
         <v>450</v>
       </c>
-      <c r="D22" s="41">
+      <c r="D22" s="40">
         <f>IF(AND(D20&gt;=1,D20&lt;=3),INT(D12&amp;1),0)</f>
         <v>0</v>
       </c>
-      <c r="E22" s="30"/>
-      <c r="F22" s="38" t="str">
+      <c r="E22" s="29"/>
+      <c r="F22" s="37" t="str">
         <f>IF(D22&gt;0,IF((COUNTIF(CTF!$C$2:$C$193,D22))=1,"RET","NOT RET"),"NONE")</f>
         <v>NONE</v>
       </c>
-      <c r="G22" s="30"/>
-      <c r="H22" s="38" t="str">
+      <c r="G22" s="29"/>
+      <c r="H22" s="37" t="str">
         <f>IF(D22&gt;0,IF(VLOOKUP(D22,CTF!$C$2:$C$193,2,FALSE),"EL","NOT EL"),"")</f>
         <v/>
       </c>
-      <c r="I22" s="33"/>
-      <c r="J22" s="27"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="26"/>
     </row>
     <row r="23" spans="3:10" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C23" s="35"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="42"/>
-      <c r="G23" s="35"/>
-      <c r="H23" s="42"/>
-      <c r="I23" s="36"/>
-      <c r="J23" s="14"/>
+      <c r="C23" s="34"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="34"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="41"/>
+      <c r="I23" s="35"/>
+      <c r="J23" s="13"/>
     </row>
     <row r="24" spans="3:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C24" s="30" t="s">
+      <c r="C24" s="29" t="s">
         <v>451</v>
       </c>
-      <c r="D24" s="41">
+      <c r="D24" s="40">
         <f>IF(AND(D20&gt;=2,D20&lt;=3),INT(D12&amp;2),0)</f>
         <v>0</v>
       </c>
-      <c r="E24" s="30"/>
-      <c r="F24" s="38" t="str">
+      <c r="E24" s="29"/>
+      <c r="F24" s="37" t="str">
         <f>IF(D24&gt;0,IF((COUNTIF(CTF!$C$2:$C$193,D24))=1,"RET","NOT RET"),"NONE")</f>
         <v>NONE</v>
       </c>
-      <c r="G24" s="30"/>
-      <c r="H24" s="38" t="str">
+      <c r="G24" s="29"/>
+      <c r="H24" s="37" t="str">
         <f>IF(D24&gt;0,IF(VLOOKUP(D24,CTF!$C$2:$C$193,2,FALSE),"EL","NOT EL"),"")</f>
         <v/>
       </c>
-      <c r="I24" s="33"/>
-      <c r="J24" s="27"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="26"/>
     </row>
     <row r="25" spans="3:10" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C25" s="35"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="35"/>
-      <c r="F25" s="42"/>
-      <c r="G25" s="35"/>
-      <c r="H25" s="42"/>
-      <c r="I25" s="36"/>
-      <c r="J25" s="14"/>
+      <c r="C25" s="34"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="41"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="41"/>
+      <c r="I25" s="35"/>
+      <c r="J25" s="13"/>
     </row>
     <row r="26" spans="3:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C26" s="30" t="s">
+      <c r="C26" s="29" t="s">
         <v>452</v>
       </c>
-      <c r="D26" s="41">
+      <c r="D26" s="40">
         <f>IF(AND(D20&gt;2,D20&lt;=3),INT(D12&amp;3),0)</f>
         <v>0</v>
       </c>
-      <c r="E26" s="30"/>
-      <c r="F26" s="38" t="str">
+      <c r="E26" s="29"/>
+      <c r="F26" s="37" t="str">
         <f>IF(D26&gt;0,IF((COUNTIF(CTF!$C$2:$C$193,D26))=1,"RET","NOT RET"),"NONE")</f>
         <v>NONE</v>
       </c>
-      <c r="G26" s="30"/>
-      <c r="H26" s="38" t="str">
+      <c r="G26" s="29"/>
+      <c r="H26" s="37" t="str">
         <f>IF(D26&gt;0,IF(VLOOKUP(D26,CTF!$C$2:$C$193,2,FALSE),"EL","NOT EL"),"")</f>
         <v/>
       </c>
-      <c r="I26" s="33"/>
-      <c r="J26" s="27"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -8031,47 +7550,47 @@
     <mergeCell ref="F6:H8"/>
   </mergeCells>
   <conditionalFormatting sqref="D8">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="notBetween">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="notBetween">
       <formula>1000</formula>
       <formula>9999</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D22">
-    <cfRule type="expression" dxfId="10" priority="8">
+    <cfRule type="expression" dxfId="8" priority="8">
       <formula>AND($F$22="RET",$H$22="EL")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D24">
-    <cfRule type="expression" dxfId="9" priority="9">
+    <cfRule type="expression" dxfId="7" priority="9">
       <formula>AND($F$24="RET",$H$24="EL")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D26">
-    <cfRule type="expression" dxfId="8" priority="10">
+    <cfRule type="expression" dxfId="6" priority="10">
       <formula>AND($F$26="RET",$H$26="EL")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F14">
-    <cfRule type="expression" dxfId="7" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>$F$14="VALID"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="7">
+    <cfRule type="expression" dxfId="4" priority="7">
       <formula>$F$14="EXPIRED"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F22 F24 F26">
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$F22="RET"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>$F22="NOT RET"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H22 H24 H26">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>$H22="EL"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="5">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>$H22="NOT EL"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8081,1190 +7600,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="B2:X19"/>
-  <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="2.69921875" customWidth="1"/>
-    <col min="2" max="2" width="4.69921875" customWidth="1"/>
-    <col min="3" max="6" width="8.3984375" customWidth="1"/>
-    <col min="7" max="7" width="3.3984375" customWidth="1"/>
-    <col min="8" max="21" width="4.296875" customWidth="1"/>
-    <col min="22" max="22" width="5.69921875" customWidth="1"/>
-    <col min="23" max="24" width="9.09765625" customWidth="1"/>
-    <col min="25" max="26" width="8" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="44" t="s">
-        <v>453</v>
-      </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
-      <c r="U2" s="3"/>
-      <c r="V2" s="43"/>
-      <c r="W2" s="3"/>
-      <c r="X2" s="3"/>
-    </row>
-    <row r="3" spans="2:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3"/>
-      <c r="V3" s="43"/>
-      <c r="W3" s="3"/>
-      <c r="X3" s="3"/>
-    </row>
-    <row r="4" spans="2:24" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="3" t="s">
-        <v>454</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3" t="s">
-        <v>455</v>
-      </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="43"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-    </row>
-    <row r="5" spans="2:24" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="45" t="s">
-        <v>456</v>
-      </c>
-      <c r="C5" s="46" t="s">
-        <v>457</v>
-      </c>
-      <c r="D5" s="46" t="s">
-        <v>458</v>
-      </c>
-      <c r="E5" s="46" t="s">
-        <v>459</v>
-      </c>
-      <c r="F5" s="47" t="s">
-        <v>460</v>
-      </c>
-      <c r="G5" s="48" t="s">
-        <v>461</v>
-      </c>
-      <c r="H5" s="49" t="s">
-        <v>462</v>
-      </c>
-      <c r="I5" s="50" t="s">
-        <v>463</v>
-      </c>
-      <c r="J5" s="50" t="s">
-        <v>464</v>
-      </c>
-      <c r="K5" s="50" t="s">
-        <v>465</v>
-      </c>
-      <c r="L5" s="50" t="s">
-        <v>466</v>
-      </c>
-      <c r="M5" s="50" t="s">
-        <v>467</v>
-      </c>
-      <c r="N5" s="50" t="s">
-        <v>468</v>
-      </c>
-      <c r="O5" s="50" t="s">
-        <v>469</v>
-      </c>
-      <c r="P5" s="50" t="s">
-        <v>470</v>
-      </c>
-      <c r="Q5" s="50" t="s">
-        <v>471</v>
-      </c>
-      <c r="R5" s="50" t="s">
-        <v>472</v>
-      </c>
-      <c r="S5" s="50" t="s">
-        <v>473</v>
-      </c>
-      <c r="T5" s="50" t="s">
-        <v>474</v>
-      </c>
-      <c r="U5" s="50" t="s">
-        <v>475</v>
-      </c>
-      <c r="V5" s="51" t="s">
-        <v>476</v>
-      </c>
-      <c r="W5" s="3"/>
-      <c r="X5" s="3"/>
-    </row>
-    <row r="6" spans="2:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="52">
-        <v>1</v>
-      </c>
-      <c r="C6" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!#REF!)="1"))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D6" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!C6:C435)="1"))</f>
-        <v>105</v>
-      </c>
-      <c r="E6" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="1"),--((CTF!#REF!)=0))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F6" s="43" t="e">
-        <f t="shared" ref="F6:F14" si="0">(C6-D6)-E6</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G6" s="53">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$2:$C$5)="2"))</f>
-        <v>1</v>
-      </c>
-      <c r="H6" s="54">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="1"),--((CTF!$C$6:$C$435)&gt;10),--((CTF!$C$6:$C$435)&lt;99))</f>
-        <v>4</v>
-      </c>
-      <c r="I6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="1"),--((CTF!$C$6:$C$435)&gt;100),--((CTF!$C$6:$C$435)&lt;999))</f>
-        <v>8</v>
-      </c>
-      <c r="J6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="1"),--((CTF!$C$6:$C$435)&gt;1000),--((CTF!$C$6:$C$435)&lt;9999))</f>
-        <v>7</v>
-      </c>
-      <c r="K6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="1"),--((CTF!$C$6:$C$435)&gt;10000),--((CTF!$C$6:$C$435)&lt;99999))</f>
-        <v>13</v>
-      </c>
-      <c r="L6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="1"),--((CTF!$C$6:$C$435)&gt;100000),--((CTF!$C$6:$C$435)&lt;999999))</f>
-        <v>18</v>
-      </c>
-      <c r="M6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="1"),--((CTF!$C$6:$C$435)&gt;1000000),--((CTF!$C$6:$C$435)&lt;9999999))</f>
-        <v>16</v>
-      </c>
-      <c r="N6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="1"),--((CTF!$C$6:$C$435)&gt;10000000),--((CTF!$C$6:$C$435)&lt;99999999))</f>
-        <v>17</v>
-      </c>
-      <c r="O6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="1"),--((CTF!$C$6:$C$435)&gt;100000000),--((CTF!$C$6:$C$435)&lt;999999999))</f>
-        <v>11</v>
-      </c>
-      <c r="P6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="1"),--((CTF!$C$6:$C$435)&gt;1000000000),--((CTF!$C$6:$C$435)&lt;9999999999))</f>
-        <v>9</v>
-      </c>
-      <c r="Q6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="1"),--((CTF!$C$6:$C$435)&gt;10000000000),--((CTF!$C$6:$C$435)&lt;99999999999))</f>
-        <v>2</v>
-      </c>
-      <c r="R6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="1"),--((CTF!$C$6:$C$193)&gt;100000000000),--((CTF!$C$6:$C$193)&lt;999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="S6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="1"),--((CTF!$C$6:$C$193)&gt;1000000000000),--((CTF!$C$6:$C$193)&lt;9999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="T6" s="55">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="1"),--((CTF!$C$6:$C$193)&gt;10000000000000),--((CTF!$C$6:$C$193)&lt;99999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="U6" s="56">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="1"),--((CTF!$C$6:$C$193)&gt;100000000000000),--((CTF!$C$6:$C$193)&lt;1000000000000000))</f>
-        <v>0</v>
-      </c>
-      <c r="V6" s="57">
-        <f t="shared" ref="V6:V14" si="1">SUM(H6:U6)</f>
-        <v>105</v>
-      </c>
-      <c r="W6" s="58"/>
-      <c r="X6" s="3"/>
-    </row>
-    <row r="7" spans="2:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="52">
-        <v>2</v>
-      </c>
-      <c r="C7" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!#REF!)="2"))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!C6:C435)="2"))</f>
-        <v>179</v>
-      </c>
-      <c r="E7" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="2"),--((CTF!#REF!)=0))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F7" s="43" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G7" s="53">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$2:$C$5)="2"))</f>
-        <v>1</v>
-      </c>
-      <c r="H7" s="59">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;10),--((CTF!$C$6:$C$435)&lt;99))</f>
-        <v>4</v>
-      </c>
-      <c r="I7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;100),--((CTF!$C$6:$C$435)&lt;999))</f>
-        <v>11</v>
-      </c>
-      <c r="J7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;1000),--((CTF!$C$6:$C$435)&lt;9999))</f>
-        <v>14</v>
-      </c>
-      <c r="K7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;10000),--((CTF!$C$6:$C$435)&lt;99999))</f>
-        <v>15</v>
-      </c>
-      <c r="L7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;100000),--((CTF!$C$6:$C$435)&lt;999999))</f>
-        <v>22</v>
-      </c>
-      <c r="M7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;1000000),--((CTF!$C$6:$C$435)&lt;9999999))</f>
-        <v>27</v>
-      </c>
-      <c r="N7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;10000000),--((CTF!$C$6:$C$435)&lt;99999999))</f>
-        <v>41</v>
-      </c>
-      <c r="O7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;100000000),--((CTF!$C$6:$C$435)&lt;999999999))</f>
-        <v>17</v>
-      </c>
-      <c r="P7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;1000000000),--((CTF!$C$6:$C$435)&lt;9999999999))</f>
-        <v>12</v>
-      </c>
-      <c r="Q7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;10000000000),--((CTF!$C$6:$C$435)&lt;99999999999))</f>
-        <v>10</v>
-      </c>
-      <c r="R7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="2"),--((CTF!$C$6:$C$193)&gt;100000000000),--((CTF!$C$6:$C$193)&lt;999999999999))</f>
-        <v>3</v>
-      </c>
-      <c r="S7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="2"),--((CTF!$C$6:$C$193)&gt;1000000000000),--((CTF!$C$6:$C$193)&lt;9999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="T7" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="2"),--((CTF!$C$6:$C$193)&gt;10000000000000),--((CTF!$C$6:$C$193)&lt;99999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="U7" s="60">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="2"),--((CTF!$C$6:$C$193)&gt;100000000000000),--((CTF!$C$6:$C$193)&lt;1000000000000000))</f>
-        <v>0</v>
-      </c>
-      <c r="V7" s="57">
-        <f t="shared" si="1"/>
-        <v>176</v>
-      </c>
-      <c r="W7" s="3"/>
-      <c r="X7" s="3"/>
-    </row>
-    <row r="8" spans="2:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="52">
-        <v>3</v>
-      </c>
-      <c r="C8" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!#REF!)="3"))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!C6:C435)="3"))</f>
-        <v>107</v>
-      </c>
-      <c r="E8" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="3"),--((CTF!#REF!)=0))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F8" s="43" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G8" s="53">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$2:$C$5)="3"))</f>
-        <v>1</v>
-      </c>
-      <c r="H8" s="59">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="3"),--((CTF!$C$6:$C$435)&gt;10),--((CTF!$C$6:$C$435)&lt;99))</f>
-        <v>5</v>
-      </c>
-      <c r="I8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="3"),--((CTF!$C$6:$C$435)&gt;100),--((CTF!$C$6:$C$435)&lt;999))</f>
-        <v>14</v>
-      </c>
-      <c r="J8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="3"),--((CTF!$C$6:$C$435)&gt;1000),--((CTF!$C$6:$C$435)&lt;9999))</f>
-        <v>18</v>
-      </c>
-      <c r="K8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="3"),--((CTF!$C$6:$C$435)&gt;10000),--((CTF!$C$6:$C$435)&lt;99999))</f>
-        <v>21</v>
-      </c>
-      <c r="L8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="3"),--((CTF!$C$6:$C$435)&gt;100000),--((CTF!$C$6:$C$435)&lt;999999))</f>
-        <v>17</v>
-      </c>
-      <c r="M8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="3"),--((CTF!$C$6:$C$435)&gt;1000000),--((CTF!$C$6:$C$435)&lt;9999999))</f>
-        <v>16</v>
-      </c>
-      <c r="N8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="3"),--((CTF!$C$6:$C$435)&gt;10000000),--((CTF!$C$6:$C$435)&lt;99999999))</f>
-        <v>6</v>
-      </c>
-      <c r="O8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="3"),--((CTF!$C$6:$C$435)&gt;100000000),--((CTF!$C$6:$C$435)&lt;999999999))</f>
-        <v>7</v>
-      </c>
-      <c r="P8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="3"),--((CTF!$C$6:$C$435)&gt;1000000000),--((CTF!$C$6:$C$435)&lt;9999999999))</f>
-        <v>3</v>
-      </c>
-      <c r="Q8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;10000000000),--((CTF!$C$6:$C$435)&lt;99999999999))</f>
-        <v>10</v>
-      </c>
-      <c r="R8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="2"),--((CTF!$C$6:$C$193)&gt;100000000000),--((CTF!$C$6:$C$193)&lt;999999999999))</f>
-        <v>3</v>
-      </c>
-      <c r="S8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="3"),--((CTF!$C$6:$C$193)&gt;1000000000000),--((CTF!$C$6:$C$193)&lt;9999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="T8" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="3"),--((CTF!$C$6:$C$193)&gt;10000000000000),--((CTF!$C$6:$C$193)&lt;99999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="U8" s="60">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="3"),--((CTF!$C$6:$C$193)&gt;100000000000000),--((CTF!$C$6:$C$193)&lt;1000000000000000))</f>
-        <v>0</v>
-      </c>
-      <c r="V8" s="57">
-        <f t="shared" si="1"/>
-        <v>120</v>
-      </c>
-      <c r="W8" s="3"/>
-      <c r="X8" s="3"/>
-    </row>
-    <row r="9" spans="2:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="52">
-        <v>4</v>
-      </c>
-      <c r="C9" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!#REF!)="4"))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!C6:C435)="4"))</f>
-        <v>39</v>
-      </c>
-      <c r="E9" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="4"),--((CTF!#REF!)=0))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F9" s="43" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G9" s="53">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$2:$C$5)="4"))</f>
-        <v>1</v>
-      </c>
-      <c r="H9" s="59">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="4"),--((CTF!$C$6:$C$435)&gt;10),--((CTF!$C$6:$C$435)&lt;99))</f>
-        <v>6</v>
-      </c>
-      <c r="I9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="4"),--((CTF!$C$6:$C$435)&gt;100),--((CTF!$C$6:$C$435)&lt;999))</f>
-        <v>7</v>
-      </c>
-      <c r="J9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="4"),--((CTF!$C$6:$C$435)&gt;1000),--((CTF!$C$6:$C$435)&lt;9999))</f>
-        <v>10</v>
-      </c>
-      <c r="K9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="4"),--((CTF!$C$6:$C$435)&gt;10000),--((CTF!$C$6:$C$435)&lt;99999))</f>
-        <v>7</v>
-      </c>
-      <c r="L9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="4"),--((CTF!$C$6:$C$435)&gt;100000),--((CTF!$C$6:$C$435)&lt;999999))</f>
-        <v>5</v>
-      </c>
-      <c r="M9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="4"),--((CTF!$C$6:$C$435)&gt;1000000),--((CTF!$C$6:$C$435)&lt;9999999))</f>
-        <v>4</v>
-      </c>
-      <c r="N9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="4"),--((CTF!$C$6:$C$435)&gt;10000000),--((CTF!$C$6:$C$435)&lt;99999999))</f>
-        <v>0</v>
-      </c>
-      <c r="O9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="4"),--((CTF!$C$6:$C$435)&gt;100000000),--((CTF!$C$6:$C$435)&lt;999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="P9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="4"),--((CTF!$C$6:$C$435)&gt;1000000000),--((CTF!$C$6:$C$435)&lt;9999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="Q9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$435)="2"),--((CTF!$C$6:$C$435)&gt;10000000000),--((CTF!$C$6:$C$435)&lt;99999999999))</f>
-        <v>10</v>
-      </c>
-      <c r="R9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="2"),--((CTF!$C$6:$C$193)&gt;100000000000),--((CTF!$C$6:$C$193)&lt;999999999999))</f>
-        <v>3</v>
-      </c>
-      <c r="S9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="4"),--((CTF!$C$6:$C$193)&gt;1000000000000),--((CTF!$C$6:$C$193)&lt;9999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="T9" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="4"),--((CTF!$C$6:$C$193)&gt;10000000000000),--((CTF!$C$6:$C$193)&lt;99999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="U9" s="60">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="4"),--((CTF!$C$6:$C$193)&gt;100000000000000),--((CTF!$C$6:$C$193)&lt;1000000000000000))</f>
-        <v>0</v>
-      </c>
-      <c r="V9" s="57">
-        <f t="shared" si="1"/>
-        <v>52</v>
-      </c>
-      <c r="W9" s="3"/>
-      <c r="X9" s="3"/>
-    </row>
-    <row r="10" spans="2:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="52">
-        <v>5</v>
-      </c>
-      <c r="C10" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!#REF!)="5"))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!C6:C249)="5"))</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="5"),--((CTF!#REF!)=0))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F10" s="43" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G10" s="53">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$2:$C$5)="5"))</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="59">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="5"),--((CTF!$C$6:$C$249)&gt;10),--((CTF!$C$6:$C$249)&lt;99))</f>
-        <v>0</v>
-      </c>
-      <c r="I10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="5"),--((CTF!$C$6:$C$249)&gt;100),--((CTF!$C$6:$C$249)&lt;999))</f>
-        <v>0</v>
-      </c>
-      <c r="J10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="5"),--((CTF!$C$6:$C$249)&gt;1000),--((CTF!$C$6:$C$249)&lt;9999))</f>
-        <v>0</v>
-      </c>
-      <c r="K10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="5"),--((CTF!$C$6:$C$249)&gt;10000),--((CTF!$C$6:$C$249)&lt;99999))</f>
-        <v>0</v>
-      </c>
-      <c r="L10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="5"),--((CTF!$C$6:$C$249)&gt;100000),--((CTF!$C$6:$C$249)&lt;999999))</f>
-        <v>0</v>
-      </c>
-      <c r="M10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="5"),--((CTF!$C$6:$C$249)&gt;1000000),--((CTF!$C$6:$C$249)&lt;9999999))</f>
-        <v>0</v>
-      </c>
-      <c r="N10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="5"),--((CTF!$C$6:$C$249)&gt;10000000),--((CTF!$C$6:$C$249)&lt;99999999))</f>
-        <v>0</v>
-      </c>
-      <c r="O10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="5"),--((CTF!$C$6:$C$193)&gt;100000000),--((CTF!$C$6:$C$193)&lt;999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="P10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="5"),--((CTF!$C$6:$C$193)&gt;1000000000),--((CTF!$C$6:$C$193)&lt;9999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="Q10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="5"),--((CTF!$C$6:$C$193)&gt;10000000000),--((CTF!$C$6:$C$193)&lt;99999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="R10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="5"),--((CTF!$C$6:$C$193)&gt;100000000000),--((CTF!$C$6:$C$193)&lt;999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="S10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="5"),--((CTF!$C$6:$C$193)&gt;1000000000000),--((CTF!$C$6:$C$193)&lt;9999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="T10" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="5"),--((CTF!$C$6:$C$193)&gt;10000000000000),--((CTF!$C$6:$C$193)&lt;99999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="U10" s="60">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="5"),--((CTF!$C$6:$C$193)&gt;100000000000000),--((CTF!$C$6:$C$193)&lt;1000000000000000))</f>
-        <v>0</v>
-      </c>
-      <c r="V10" s="57">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="W10" s="3"/>
-      <c r="X10" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="2:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="52">
-        <v>6</v>
-      </c>
-      <c r="C11" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!#REF!)="6"))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!C6:C249)="6"))</f>
-        <v>0</v>
-      </c>
-      <c r="E11" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="6"),--((CTF!#REF!)=0))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F11" s="43" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G11" s="53">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$2:$C$5)="6"))</f>
-        <v>0</v>
-      </c>
-      <c r="H11" s="59">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="6"),--((CTF!$C$6:$C$249)&gt;10),--((CTF!$C$6:$C$249)&lt;99))</f>
-        <v>0</v>
-      </c>
-      <c r="I11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="6"),--((CTF!$C$6:$C$249)&gt;100),--((CTF!$C$6:$C$249)&lt;999))</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="6"),--((CTF!$C$6:$C$249)&gt;1000),--((CTF!$C$6:$C$249)&lt;9999))</f>
-        <v>0</v>
-      </c>
-      <c r="K11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="6"),--((CTF!$C$6:$C$249)&gt;10000),--((CTF!$C$6:$C$249)&lt;99999))</f>
-        <v>0</v>
-      </c>
-      <c r="L11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="6"),--((CTF!$C$6:$C$249)&gt;100000),--((CTF!$C$6:$C$249)&lt;999999))</f>
-        <v>0</v>
-      </c>
-      <c r="M11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="6"),--((CTF!$C$6:$C$249)&gt;1000000),--((CTF!$C$6:$C$249)&lt;9999999))</f>
-        <v>0</v>
-      </c>
-      <c r="N11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="6"),--((CTF!$C$6:$C$249)&gt;10000000),--((CTF!$C$6:$C$249)&lt;99999999))</f>
-        <v>0</v>
-      </c>
-      <c r="O11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="6"),--((CTF!$C$6:$C$193)&gt;100000000),--((CTF!$C$6:$C$193)&lt;999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="P11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="6"),--((CTF!$C$6:$C$193)&gt;1000000000),--((CTF!$C$6:$C$193)&lt;9999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="Q11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="6"),--((CTF!$C$6:$C$193)&gt;10000000000),--((CTF!$C$6:$C$193)&lt;99999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="R11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="6"),--((CTF!$C$6:$C$193)&gt;100000000000),--((CTF!$C$6:$C$193)&lt;999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="S11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="6"),--((CTF!$C$6:$C$193)&gt;1000000000000),--((CTF!$C$6:$C$193)&lt;9999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="T11" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="6"),--((CTF!$C$6:$C$193)&gt;10000000000000),--((CTF!$C$6:$C$193)&lt;99999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="U11" s="60">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="6"),--((CTF!$C$6:$C$193)&gt;100000000000000),--((CTF!$C$6:$C$193)&lt;1000000000000000))</f>
-        <v>0</v>
-      </c>
-      <c r="V11" s="57">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="W11" s="3"/>
-      <c r="X11" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="2:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="52">
-        <v>7</v>
-      </c>
-      <c r="C12" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!#REF!)="7"))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!C6:C193)="7"))</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="7"),--((CTF!#REF!)=0))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F12" s="43" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G12" s="53">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$2:$C$5)="7"))</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="59">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="7"),--((CTF!$C$6:$C$193)&gt;10),--((CTF!$C$6:$C$193)&lt;99))</f>
-        <v>0</v>
-      </c>
-      <c r="I12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="7"),--((CTF!$C$6:$C$249)&gt;100),--((CTF!$C$6:$C$249)&lt;999))</f>
-        <v>0</v>
-      </c>
-      <c r="J12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="7"),--((CTF!$C$6:$C$193)&gt;1000),--((CTF!$C$6:$C$193)&lt;9999))</f>
-        <v>0</v>
-      </c>
-      <c r="K12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="7"),--((CTF!$C$6:$C$249)&gt;10000),--((CTF!$C$6:$C$249)&lt;99999))</f>
-        <v>0</v>
-      </c>
-      <c r="L12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="7"),--((CTF!$C$6:$C$193)&gt;100000),--((CTF!$C$6:$C$193)&lt;999999))</f>
-        <v>0</v>
-      </c>
-      <c r="M12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="7"),--((CTF!$C$6:$C$249)&gt;1000000),--((CTF!$C$6:$C$249)&lt;9999999))</f>
-        <v>0</v>
-      </c>
-      <c r="N12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="7"),--((CTF!$C$6:$C$193)&gt;10000000),--((CTF!$C$6:$C$193)&lt;99999999))</f>
-        <v>0</v>
-      </c>
-      <c r="O12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="7"),--((CTF!$C$6:$C$193)&gt;100000000),--((CTF!$C$6:$C$193)&lt;999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="P12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="7"),--((CTF!$C$6:$C$193)&gt;1000000000),--((CTF!$C$6:$C$193)&lt;9999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="Q12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="7"),--((CTF!$C$6:$C$193)&gt;10000000000),--((CTF!$C$6:$C$193)&lt;99999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="R12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="7"),--((CTF!$C$6:$C$193)&gt;100000000000),--((CTF!$C$6:$C$193)&lt;999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="S12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="7"),--((CTF!$C$6:$C$193)&gt;1000000000000),--((CTF!$C$6:$C$193)&lt;9999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="T12" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="7"),--((CTF!$C$6:$C$193)&gt;10000000000000),--((CTF!$C$6:$C$193)&lt;99999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="U12" s="60">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="7"),--((CTF!$C$6:$C$193)&gt;100000000000000),--((CTF!$C$6:$C$193)&lt;1000000000000000))</f>
-        <v>0</v>
-      </c>
-      <c r="V12" s="57">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="W12" s="3"/>
-      <c r="X12" s="3"/>
-    </row>
-    <row r="13" spans="2:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="52">
-        <v>8</v>
-      </c>
-      <c r="C13" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!#REF!)="8"))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!C6:C193)="8"))</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="43" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="8"),--((CTF!#REF!)=0))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F13" s="43" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G13" s="53">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$2:$C$5)="8"))</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="59">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;10),--((CTF!$C$6:$C$193)&lt;99))</f>
-        <v>0</v>
-      </c>
-      <c r="I13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;100),--((CTF!$C$6:$C$193)&lt;999))</f>
-        <v>0</v>
-      </c>
-      <c r="J13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;1000),--((CTF!$C$6:$C$193)&lt;9999))</f>
-        <v>0</v>
-      </c>
-      <c r="K13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;10000),--((CTF!$C$6:$C$193)&lt;99999))</f>
-        <v>0</v>
-      </c>
-      <c r="L13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;100000),--((CTF!$C$6:$C$193)&lt;999999))</f>
-        <v>0</v>
-      </c>
-      <c r="M13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;1000000),--((CTF!$C$6:$C$193)&lt;9999999))</f>
-        <v>0</v>
-      </c>
-      <c r="N13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;10000000),--((CTF!$C$6:$C$193)&lt;99999999))</f>
-        <v>0</v>
-      </c>
-      <c r="O13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;100000000),--((CTF!$C$6:$C$193)&lt;999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="P13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;1000000000),--((CTF!$C$6:$C$193)&lt;9999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="Q13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;10000000000),--((CTF!$C$6:$C$193)&lt;99999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="R13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;100000000000),--((CTF!$C$6:$C$193)&lt;999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="S13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;1000000000000),--((CTF!$C$6:$C$193)&lt;9999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="T13" s="43">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;10000000000000),--((CTF!$C$6:$C$193)&lt;99999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="U13" s="60">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="8"),--((CTF!$C$6:$C$193)&gt;100000000000000),--((CTF!$C$6:$C$193)&lt;1000000000000000))</f>
-        <v>0</v>
-      </c>
-      <c r="V13" s="57">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="W13" s="3"/>
-      <c r="X13" s="3"/>
-    </row>
-    <row r="14" spans="2:24" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="61">
-        <v>9</v>
-      </c>
-      <c r="C14" s="62" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!#REF!)="9"))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!C6:C187)="9"))</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="62" t="e">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$249)="9"),--((CTF!#REF!)=0))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F14" s="63" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$2:$C$5)="9"))</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="64">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;10),--((CTF!$C$6:$C$193)&lt;99))</f>
-        <v>0</v>
-      </c>
-      <c r="I14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;100),--((CTF!$C$6:$C$193)&lt;999))</f>
-        <v>0</v>
-      </c>
-      <c r="J14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;1000),--((CTF!$C$6:$C$193)&lt;9999))</f>
-        <v>0</v>
-      </c>
-      <c r="K14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;10000),--((CTF!$C$6:$C$193)&lt;99999))</f>
-        <v>0</v>
-      </c>
-      <c r="L14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;100000),--((CTF!$C$6:$C$193)&lt;999999))</f>
-        <v>0</v>
-      </c>
-      <c r="M14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;1000000),--((CTF!$C$6:$C$193)&lt;9999999))</f>
-        <v>0</v>
-      </c>
-      <c r="N14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;10000000),--((CTF!$C$6:$C$193)&lt;99999999))</f>
-        <v>0</v>
-      </c>
-      <c r="O14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;100000000),--((CTF!$C$6:$C$193)&lt;999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="P14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;1000000000),--((CTF!$C$6:$C$193)&lt;9999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="Q14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;10000000000),--((CTF!$C$6:$C$193)&lt;99999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="R14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;100000000000),--((CTF!$C$6:$C$193)&lt;999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="S14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;1000000000000),--((CTF!$C$6:$C$193)&lt;9999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="T14" s="62">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;10000000000000),--((CTF!$C$6:$C$193)&lt;99999999999999))</f>
-        <v>0</v>
-      </c>
-      <c r="U14" s="63">
-        <f>SUMPRODUCT(--(LEFT(CTF!$C$6:$C$193)="9"),--((CTF!$C$6:$C$193)&gt;100000000000000),--((CTF!$C$6:$C$193)&lt;1000000000000000))</f>
-        <v>0</v>
-      </c>
-      <c r="V14" s="65">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="W14" s="3"/>
-      <c r="X14" s="3"/>
-    </row>
-    <row r="15" spans="2:24" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="66"/>
-      <c r="C15" s="67" t="e">
-        <f t="shared" ref="C15:F15" si="2">SUM(C6:C14)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D15" s="67">
-        <f t="shared" si="2"/>
-        <v>430</v>
-      </c>
-      <c r="E15" s="68" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-      <c r="F15" s="68" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G15" s="66"/>
-      <c r="H15" s="69">
-        <f t="shared" ref="H15:V15" si="3">SUM(H6:H14)</f>
-        <v>19</v>
-      </c>
-      <c r="I15" s="69">
-        <f t="shared" si="3"/>
-        <v>40</v>
-      </c>
-      <c r="J15" s="69">
-        <f t="shared" si="3"/>
-        <v>49</v>
-      </c>
-      <c r="K15" s="69">
-        <f t="shared" si="3"/>
-        <v>56</v>
-      </c>
-      <c r="L15" s="69">
-        <f t="shared" si="3"/>
-        <v>62</v>
-      </c>
-      <c r="M15" s="69">
-        <f t="shared" si="3"/>
-        <v>63</v>
-      </c>
-      <c r="N15" s="69">
-        <f t="shared" si="3"/>
-        <v>64</v>
-      </c>
-      <c r="O15" s="69">
-        <f t="shared" si="3"/>
-        <v>35</v>
-      </c>
-      <c r="P15" s="69">
-        <f t="shared" si="3"/>
-        <v>24</v>
-      </c>
-      <c r="Q15" s="69">
-        <f t="shared" si="3"/>
-        <v>32</v>
-      </c>
-      <c r="R15" s="69">
-        <f t="shared" si="3"/>
-        <v>9</v>
-      </c>
-      <c r="S15" s="69">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="T15" s="69">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="U15" s="69">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="V15" s="70">
-        <f t="shared" si="3"/>
-        <v>453</v>
-      </c>
-      <c r="W15" s="3"/>
-      <c r="X15" s="3"/>
-    </row>
-    <row r="17" spans="3:23" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="3"/>
-      <c r="S17" s="3"/>
-      <c r="T17" s="3"/>
-      <c r="U17" s="3"/>
-      <c r="V17" s="43"/>
-      <c r="W17" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="3:23" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C18" s="97" t="s">
-        <v>477</v>
-      </c>
-      <c r="D18" s="98"/>
-      <c r="E18" s="71" t="e">
-        <f>D15-E15</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="G18" s="3"/>
-      <c r="H18" s="72">
-        <f>10*3</f>
-        <v>30</v>
-      </c>
-      <c r="I18" s="72">
-        <f t="shared" ref="I18:O18" si="4">+H18*3</f>
-        <v>90</v>
-      </c>
-      <c r="J18" s="72">
-        <f t="shared" si="4"/>
-        <v>270</v>
-      </c>
-      <c r="K18" s="72">
-        <f t="shared" si="4"/>
-        <v>810</v>
-      </c>
-      <c r="L18" s="72">
-        <f t="shared" si="4"/>
-        <v>2430</v>
-      </c>
-      <c r="M18" s="72">
-        <f t="shared" si="4"/>
-        <v>7290</v>
-      </c>
-      <c r="N18" s="72">
-        <f t="shared" si="4"/>
-        <v>21870</v>
-      </c>
-      <c r="O18" s="72">
-        <f t="shared" si="4"/>
-        <v>65610</v>
-      </c>
-      <c r="P18" s="73"/>
-      <c r="Q18" s="73"/>
-      <c r="R18" s="73"/>
-      <c r="S18" s="73"/>
-      <c r="T18" s="73"/>
-      <c r="U18" s="73"/>
-      <c r="V18" s="43"/>
-      <c r="W18" s="3"/>
-    </row>
-    <row r="19" spans="3:23" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="97" t="s">
-        <v>478</v>
-      </c>
-      <c r="D19" s="98"/>
-      <c r="E19" s="71" t="e">
-        <f>E15</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="72">
-        <f t="shared" ref="H19:O19" si="5">+H18-H15</f>
-        <v>11</v>
-      </c>
-      <c r="I19" s="72">
-        <f t="shared" si="5"/>
-        <v>50</v>
-      </c>
-      <c r="J19" s="72">
-        <f t="shared" si="5"/>
-        <v>221</v>
-      </c>
-      <c r="K19" s="72">
-        <f t="shared" si="5"/>
-        <v>754</v>
-      </c>
-      <c r="L19" s="72">
-        <f t="shared" si="5"/>
-        <v>2368</v>
-      </c>
-      <c r="M19" s="72">
-        <f t="shared" si="5"/>
-        <v>7227</v>
-      </c>
-      <c r="N19" s="72">
-        <f t="shared" si="5"/>
-        <v>21806</v>
-      </c>
-      <c r="O19" s="72">
-        <f t="shared" si="5"/>
-        <v>65575</v>
-      </c>
-      <c r="P19" s="73"/>
-      <c r="Q19" s="73"/>
-      <c r="R19" s="73"/>
-      <c r="S19" s="73"/>
-      <c r="T19" s="73"/>
-      <c r="U19" s="73"/>
-      <c r="V19" s="43"/>
-      <c r="W19" s="3"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-  </mergeCells>
-  <conditionalFormatting sqref="C6:F14 H6:V14 G14">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G6:G13">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
-  <legacyDrawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="C2:E9"/>
   <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -9278,54 +7613,54 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="99" t="s">
-        <v>479</v>
-      </c>
-      <c r="D2" s="100"/>
-      <c r="E2" s="101"/>
+      <c r="C2" s="65" t="s">
+        <v>453</v>
+      </c>
+      <c r="D2" s="66"/>
+      <c r="E2" s="67"/>
     </row>
     <row r="3" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="102"/>
-      <c r="D3" s="103"/>
-      <c r="E3" s="104"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="70"/>
     </row>
     <row r="4" spans="3:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
     </row>
     <row r="5" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="75"/>
-      <c r="D5" s="76"/>
-      <c r="E5" s="77"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="45"/>
     </row>
     <row r="6" spans="3:5" ht="135.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="78"/>
-      <c r="D6" s="79" t="s">
-        <v>480</v>
-      </c>
-      <c r="E6" s="80"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="E6" s="48"/>
     </row>
     <row r="7" spans="3:5" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="78"/>
-      <c r="D7" s="81" t="s">
-        <v>481</v>
-      </c>
-      <c r="E7" s="80"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="49" t="s">
+        <v>455</v>
+      </c>
+      <c r="E7" s="48"/>
     </row>
     <row r="8" spans="3:5" ht="105.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C8" s="78"/>
-      <c r="D8" s="81" t="s">
-        <v>482</v>
-      </c>
-      <c r="E8" s="80"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="49" t="s">
+        <v>456</v>
+      </c>
+      <c r="E8" s="48"/>
     </row>
     <row r="9" spans="3:5" ht="62.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="78"/>
-      <c r="D9" s="82" t="s">
-        <v>483</v>
-      </c>
-      <c r="E9" s="80"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="50" t="s">
+        <v>457</v>
+      </c>
+      <c r="E9" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>